<commit_message>
docs: correct tracker totals and snapshot metadata
</commit_message>
<xml_diff>
--- a/TASK_TRACKER.xlsx
+++ b/TASK_TRACKER.xlsx
@@ -602,7 +602,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -619,7 +619,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Recovered 2026-07-21 from the complete v3.66.539 canonical pack and reconciled through current v3.66.811 OPV work. TASK_TRACKER_DATA.json is canonical; TASK_TRACKER.md and TASK_TRACKER.xlsx are generated from it.</t>
+          <t>Recovered 2026-07-21 from the complete v3.66.539 canonical pack and reconciled against v3.66.811 OPV evidence available on 2026-07-21. TASK_TRACKER_DATA.json is canonical; TASK_TRACKER.md and TASK_TRACKER.xlsx are generated from it.</t>
         </is>
       </c>
     </row>
@@ -661,59 +661,79 @@
         <v>269</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Decided against</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>11</v>
+      </c>
+    </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Grand total</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>Incomplete by Sandbox-able?</t>
         </is>
       </c>
-      <c r="B9" s="4" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="B11" s="4" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>Yes (source review)</t>
         </is>
       </c>
-      <c r="B10" s="6" t="n">
+      <c r="B12" s="6" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>Incomplete by Tier</t>
         </is>
       </c>
-      <c r="B12" s="4" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="B14" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="B14" s="4" t="n"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="B15" s="6" t="n">
+      <c r="B17" s="6" t="n">
         <v>1</v>
       </c>
     </row>
@@ -10641,7 +10661,7 @@
       </c>
       <c r="C269" s="13" t="inlineStr">
         <is>
-          <t>B2 override-extraction live verify -- unreviewed draft -&gt; one real download + 4 invariants (I1 not-enabled, I2 override-branch, I3 no-persist, I4 challenge-&gt;manual-handoff)</t>
+          <t>B2 override-extraction acceptance -- unreviewed draft -&gt; one real download (I1-I3 live; I4 manual-handoff inheritance source-confirmed)</t>
         </is>
       </c>
       <c r="D269" s="13" t="inlineStr">
@@ -10656,7 +10676,7 @@
       </c>
       <c r="F269" s="13" t="inlineStr">
         <is>
-          <t>Repository commit 16303769dbbdc60ba7ec40db72ca65803cda3204 records the live runner/browser probe: exactly 262,144 bytes of sanctioned video/mp4 sampled with persist=false, no file saved, the draft left review-only, draft/reviewed/config hashes restored, and all temporary state removed. The consolidated pre-merge acceptance snapshot is reports/OPV_VALIDATION_REPORT_2026-07-21.md.</t>
+          <t>Repository commit 16303769dbbdc60ba7ec40db72ca65803cda3204 records the live runner/browser probe: exactly 262,144 bytes of sanctioned video/mp4 sampled with persist=false, no file saved, the draft left review-only, draft/reviewed/config hashes restored, and all temporary state removed. That live arm demonstrated I1/I2/I3. I4 was source-confirmed, not live-triggered, because the sanctioned fixture encountered no challenge; the separate P3-T12-CALLSITE real challenge detect-to-handoff observation remains awaiting operator. The consolidated pre-merge acceptance snapshot is reports/OPV_VALIDATION_REPORT_2026-07-21.md.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Complete OPV validation hardening
</commit_message>
<xml_diff>
--- a/TASK_TRACKER.xlsx
+++ b/TASK_TRACKER.xlsx
@@ -14,8 +14,8 @@
     <sheet name="Decided against" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Awaiting operator'!$A$1:$H$22</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Completed'!$A$1:$F$273</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Awaiting operator'!$A$1:$H$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Completed'!$A$1:$F$284</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Decided against'!$A$1:$F$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -77,7 +77,7 @@
       <color rgb="00475569"/>
     </font>
   </fonts>
-  <fills count="14">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -136,11 +136,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FAE8FF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00EEF1F6"/>
       </patternFill>
     </fill>
@@ -167,7 +162,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -208,10 +203,10 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -226,10 +221,7 @@
     <xf numFmtId="0" fontId="7" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -644,7 +636,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>21</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7">
@@ -654,7 +646,7 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>272</v>
+        <v>283</v>
       </c>
     </row>
     <row r="8">
@@ -674,7 +666,7 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>304</v>
+        <v>305</v>
       </c>
     </row>
     <row r="11">
@@ -772,7 +764,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -860,857 +852,437 @@
       </c>
       <c r="G2" s="8" t="inlineStr">
         <is>
-          <t>P4</t>
+          <t>Operator-owned MOD3 target/DSN + live shadow observability + cutover + &gt;=2-week soak</t>
         </is>
       </c>
       <c r="H2" s="8" t="inlineStr">
         <is>
-          <t>Calendar/operator-bound</t>
+          <t>The MOD3 cutover/rollback mechanism is complete @804, but it is default-OFF and tests explicitly preserve this real exit criterion. Read-only readiness audit 2026-07-22: stash has a non-empty 23-row SQLite source, psycopg, and running candidate Postgres containers, but the service has no MOD3 DSN, shadow-read, or cutover enabled; neither container is yet operator-authorized. Live shadow counters are process-local and no in-process status surface currently exposes the comparison denominator, so a separate Python preflight would not attest the running service. No clock started. Select/provision the target, add secret-free in-process stats/preflight evidence, pass rehearsal and live preflight, perform the authorized cutover, run the full on-stash suite green post-cutover, then retain &gt;=336 hours of operator-soak evidence. Exact preflight, rollback, and soak checklist: reports/OPV_EXIT3_F31_READINESS_AUDIT_2026-07-22.md.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="11" t="inlineStr">
         <is>
-          <t>F0.4</t>
+          <t>OPV-F3.1</t>
         </is>
       </c>
       <c r="B3" s="12" t="inlineStr">
         <is>
-          <t>Track-F</t>
+          <t>Operator verify</t>
         </is>
       </c>
       <c r="C3" s="12" t="inlineStr">
         <is>
-          <t>WSGI fact-check -&gt; swap to waitress (systemd ExecStart edit)</t>
-        </is>
-      </c>
-      <c r="D3" s="12" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E3" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>F3.1 enqueue lane — saved search action=enqueue -&gt; cap+gates+dedup over a week</t>
+        </is>
+      </c>
+      <c r="D3" s="13" t="inlineStr">
+        <is>
+          <t>AWAITING OPERATOR (week-long live verify)</t>
+        </is>
+      </c>
+      <c r="E3" s="14" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="F3" s="10" t="inlineStr">
         <is>
-          <t>No (operator)</t>
+          <t>No (live week)</t>
         </is>
       </c>
       <c r="G3" s="12" t="inlineStr">
         <is>
-          <t>SSE --threads sizing Q</t>
+          <t>Operator-approved sanctioned rule + seven uninterrupted days</t>
         </is>
       </c>
       <c r="H3" s="12" t="inlineStr">
         <is>
-          <t>Pure systemd edit + offline waitress wheel; confirm /api/stream long-poll threads fit --threads first</t>
+          <t>LIVE @223; scheduler blocker cleared @461; time-warp/leak-freedom sandbox proof completed @539. Read-only readiness audit 2026-07-22 found the scheduler healthy (`saved_searches.run_due` enabled, 300-second task interval, last status ok) but zero saved-search rules, so no seven-day clock started. Operator must approve a bounded action=enqueue rule (hourly recommended), then preserve &gt;=168 hours of cap, downstream-gate, dedup, scheduler, and queue evidence. Exact rule fields and observation checklist: reports/OPV_EXIT3_F31_READINESS_AUDIT_2026-07-22.md. The deferred SPA action-picker tail remains part of this row. Consolidates former duplicate F3.1-WK.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>F2-HYG</t>
+          <t>CAP-ROBUST</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>Operator F2</t>
+          <t>Capture core (held-open) — anti-bot resilience</t>
         </is>
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
-          <t>Remove raw .wacz twins before sharing (7 in redacted_captures_keep.zip + the out.zip RAW set); re-scrub tiny4k SigV4 twins; ~15 x-forwarded-for files</t>
-        </is>
-      </c>
-      <c r="D4" s="8" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="E4" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F4" s="10" t="inlineStr">
-        <is>
-          <t>No (operator)</t>
+          <t>Held-open capture died on anti-bot sites before the operator could act, and a login redirect dropped the deep URL onto home. A) page-death recovery; B) 'Go to my URL' re-nav; C) challenge settle.</t>
+        </is>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
+        <is>
+          <t>LIVE A/B PASSED; challenge C pending</t>
+        </is>
+      </c>
+      <c r="E4" s="15" t="inlineStr">
+        <is>
+          <t>B (DECLARED guard change: tools/capture_session.py)</t>
+        </is>
+      </c>
+      <c r="F4" s="16" t="inlineStr">
+        <is>
+          <t>Partial (decision logic sandbox-tested; live reopen/re-nav/challenge-wait stash-only)</t>
         </is>
       </c>
       <c r="G4" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>real live challenge settle/resume acceptance</t>
         </is>
       </c>
       <c r="H4" s="8" t="inlineStr">
         <is>
-          <t>Local-only F2 hygiene; not retroactive via code</t>
+          <t>BUILT @293 with RED-first test_capture_robustness 12/12 + test_capture_goto_renav 4/4. LIVE @817: A passed when closing the active page caused the held-open runner to recover by opening a replacement page; B passed when the GOTO sentinel was consumed and navigation returned from the IANA page to example.com. These observations validate page-death recovery and operator re-navigation on stash. C remains open: exercise the challenge settle/handoff path through detector-gated resume before closure.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
         <is>
-          <t>OPV-F1.3</t>
+          <t>JW-TMPL</t>
         </is>
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>Operator verify</t>
+          <t>Recognizer / auto-template robustness</t>
         </is>
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>F1.3 cookie_admission_enabled — lapsed jar -&gt; cookies_expired (no spawn) + self-resolve</t>
+          <t>Auto-template for signed JWPlayer behind akamai/cloudflare was always weak (signed direct-media -&gt; no row selectors, 1 net pattern). Recognize the signed-media + JWPlayer shape so the draft is usable.</t>
         </is>
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
-          <t>AWAITING OPERATOR (live enablement check)</t>
-        </is>
-      </c>
-      <c r="E5" s="14" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="F5" s="10" t="inlineStr">
-        <is>
-          <t>No (live jar)</t>
+          <t>BUILT @293; SANDBOX-VERIFIED on real WACZ @298 (corpus); live-on-stash creds pending</t>
+        </is>
+      </c>
+      <c r="E5" s="17" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="F5" s="18" t="inlineStr">
+        <is>
+          <t>Yes (recognizer unit-tested on synthetic network_log; real WACZ stash-only)</t>
         </is>
       </c>
       <c r="G5" s="12" t="inlineStr">
         <is>
-          <t>login-gated site with an aged cookie jar</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H5" s="12" t="inlineStr">
         <is>
-          <t>LIVE @217 and sandbox-verified @539. On stash, set cookie_file + cookie_admission_enabled for a sanctioned login-gated site, fully lapse the jar, confirm cookies_expired prevents a worker spawn, then refresh the jar and confirm self-resolution. Consolidates former duplicate F1.3-EN.</t>
+          <t>Now verified on REAL signed-JWPlayer WACZ via the §9 corpus (reptyle/ultra/wow=wowgirls -&gt; signed_generic_token/jwplayer/pick_test_promote = R5 signing-free pattern). Remaining: live capture on stash with ultrafilms creds ('site Ultra missing password'), then flip -&gt;LIVE.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>OPV-F1.4</t>
+          <t>LOGIN-NSTEP</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>Operator verify</t>
+          <t>Capture frontier</t>
         </is>
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>F1.4 predictive_relogin on a churn-prone site -&gt; relogin at ~0.8*median</t>
-        </is>
-      </c>
-      <c r="D6" s="13" t="inlineStr">
-        <is>
-          <t>AWAITING OPERATOR (live enablement check)</t>
-        </is>
-      </c>
-      <c r="E6" s="15" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="F6" s="10" t="inlineStr">
-        <is>
-          <t>No (live churn site)</t>
+          <t>Cross-origin N-step login flow (general): plan_login_flow derivation + replay_saved_login_flow drive</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>BUILT @302 (code LIVE; live cross-origin DRIVE = operator-verify)</t>
+        </is>
+      </c>
+      <c r="E6" s="19" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F6" s="16" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
       <c r="G6" s="8" t="inlineStr">
         <is>
-          <t>sanctioned churn-prone site with at least 3 observations</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H6" s="8" t="inlineStr">
         <is>
-          <t>LIVE @218 and sandbox-verified @539. Enable predictive_relogin_enabled on a sanctioned churn-prone site with &gt;=3 observations and confirm relogin occurs at approximately 0.8 * learned median rather than the fixed 168-hour age. Consolidates former duplicate F1.4-EN.</t>
+          <t>login_flow_recorder.plan_login_flow derives a general N-step plan (type/click + await_url at each origin hop; single-origin = no await; credential resolves to a VAULT MARKER, never the secret, F2). replay_saved_login_flow drives it before the single-form cascade. Recorder/replay substrate (login_flow_recorder/macro_recorder/macro_replay) extended. Derivation unit-tested offline (test_v3_66_302_login_flow_nstep); live cross-origin browser drive is operator-verify on stash. FUNCTION_INDEX + DEPENDENCY_GRAPH regenerated. | Progress: 353 added staged 2-step login fill; 381 login_assist infers N-step (assist-only, cannot persist creds/enable host). Full cross-origin flow still needs operator live-verify.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="11" t="inlineStr">
         <is>
-          <t>OPV-F3.1</t>
+          <t>P3-T12-CALLSITE</t>
         </is>
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Operator verify</t>
+          <t>Migration Phase 3-4 / capture frontier</t>
         </is>
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
-          <t>F3.1 enqueue lane — saved search action=enqueue -&gt; cap+gates+dedup over a week</t>
+          <t>Held-open runner call-site swap (capture_session.py) to invoke the @389 challenge seam, + on-stash live real-challenge validation before any ratchet</t>
         </is>
       </c>
       <c r="D7" s="13" t="inlineStr">
         <is>
-          <t>AWAITING OPERATOR (week-long live verify)</t>
-        </is>
-      </c>
-      <c r="E7" s="14" t="inlineStr">
-        <is>
-          <t>C</t>
+          <t>LIVE detect/pause/handoff observed; detector-gated resume pending</t>
+        </is>
+      </c>
+      <c r="E7" s="19" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
       <c r="F7" s="10" t="inlineStr">
         <is>
-          <t>No (live week)</t>
+          <t>No (build+deploy DONE @458; live real-challenge on stash)</t>
         </is>
       </c>
       <c r="G7" s="12" t="inlineStr">
         <is>
-          <t>operator stash and elapsed time</t>
+          <t>human clears a real challenge so detector-gated resume can be observed</t>
         </is>
       </c>
       <c r="H7" s="12" t="inlineStr">
         <is>
-          <t>LIVE @223; scheduler blocker cleared @461; time-warp/leak-freedom sandbox proof completed @539. Create a saved-search enqueue rule and confirm caps, gates, and dedup over an uninterrupted week. The deferred SPA action-picker tail remains part of this row. Consolidates former duplicate F3.1-WK.</t>
+          <t>SHIPPED @458: the held-open runner routes challenge settle through bulk_downloader.session_capture.handle_challenge_on_page with passive-budget parity, secret-free logging, operator instructions, and no solving. LIVE @817 on the real Reptyle Cloudflare login wall: the detector recognized the challenge, paused capture, routed to operator handoff, and retained solved=false. This proves the real detect-&gt;pause-&gt;handoff half. Keep the row open until a human clears a real challenge and the detector observes it gone before resume; never infer solved from the handoff itself.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>OPV-F3.2</t>
+          <t>RPTYL</t>
         </is>
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Operator verify</t>
+          <t>Capture frontier</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>F3.2 drift-&gt;AI repair — wire stash dom_provider; enable; confirm a drift -&gt; draft_review_required</t>
+          <t>reptyle real-Chrome authenticated-profile capture (success = api_patterns &gt;= 1)</t>
         </is>
       </c>
       <c r="D8" s="13" t="inlineStr">
         <is>
-          <t>AWAITING OPERATOR (live daily-run verify)</t>
-        </is>
-      </c>
-      <c r="E8" s="16" t="inlineStr">
-        <is>
-          <t>B</t>
+          <t>AWAITING OPERATOR -- real-Chrome stash capture (no sandbox build)</t>
+        </is>
+      </c>
+      <c r="E8" s="20" t="inlineStr">
+        <is>
+          <t>M</t>
         </is>
       </c>
       <c r="F8" s="10" t="inlineStr">
         <is>
-          <t>No (stash/live AI)</t>
+          <t>No (real Chrome on stash)</t>
         </is>
       </c>
       <c r="G8" s="8" t="inlineStr">
         <is>
-          <t>sanctioned live stale site plus live AI provider</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H8" s="8" t="inlineStr">
         <is>
-          <t>Shipped @224; review-only proposal path sandbox-verified @539. The v3.66.817 safe OPV exercised enable/revert and preserved the last-run record, but a real scheduled daily repair remains. Enable automation.drift_repair_enabled (or Run-now with force) against a sanctioned stale site, confirm a draft_review_required repair and persisted last-run update. Consolidates former duplicate F3.2-LIVE.</t>
+          <t>Run the authenticated-profile capture on stash and require api_patterns &gt;= 1. The default-ON live HUD is complete and available for guided capture, so it is no longer a blocker; this row remains open solely for the real authenticated Reptyle capture and evidence review.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="11" t="inlineStr">
         <is>
-          <t>CAP-ROBUST</t>
+          <t>FR-A6.2</t>
         </is>
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>Capture core (held-open) — anti-bot resilience</t>
+          <t>Capture frontier</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>Held-open capture died on anti-bot sites before the operator could act, and a login redirect dropped the deep URL onto home. A) page-death recovery; B) 'Go to my URL' re-nav; C) challenge settle.</t>
-        </is>
-      </c>
-      <c r="D9" s="13" t="inlineStr">
-        <is>
-          <t>BUILT @293 (live-verify pending)</t>
-        </is>
-      </c>
-      <c r="E9" s="14" t="inlineStr">
-        <is>
-          <t>B (DECLARED guard change: tools/capture_session.py)</t>
-        </is>
-      </c>
-      <c r="F9" s="17" t="inlineStr">
-        <is>
-          <t>Partial (decision logic sandbox-tested; live reopen/re-nav/challenge-wait stash-only)</t>
+          <t>Builder enrichment slice 2 (non-CF / non-video.js breadth)</t>
+        </is>
+      </c>
+      <c r="D9" s="21" t="inlineStr">
+        <is>
+          <t>AWAITING OPERATOR CAPTURE DATA -- corpus-blocked (build resumes after capture)</t>
+        </is>
+      </c>
+      <c r="E9" s="20" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F9" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G9" s="12" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>corpus breadth</t>
         </is>
       </c>
       <c r="H9" s="12" t="inlineStr">
         <is>
-          <t>DONE in sandbox @293: A=per-tick reopen+re-nav-to-start_url when no live page; B=GOTO sentinel + cockpit_core.goto_capture + POST /cockpit/api/captures/goto + SPA 'Go to my URL'; C=_settle_through_challenge (BD_CHALLENGE_WAIT_S default 20, zero-cost on normal sites). GUARD capture_session.py declared fff3e972-&gt;707dcd2b; other 6 byte-identical. RED-first test_capture_robustness 12/12 + test_capture_goto_renav 4/4. Live behavior stash-only.</t>
+          <t>The recognizers already implement radiant_media_player, clappr, dashjs, youtube, jplayer, mux_hosted, and brid_tv, with synthetic detection tests; v3.66.681 also added synthetic corpus fixtures for clappr and dashjs. What remains is real guided-capture corpus evidence and builder/template enrichment for these families, not first-time recognizer implementation. Capture representative sanctioned pages with the now-complete HUD, scrub the WACZ artifacts, pin real verdicts, then resume the builder slice.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>JW-TMPL</t>
+          <t>FR-A6.3</t>
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>Recognizer / auto-template robustness</t>
+          <t>Capture frontier</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>Auto-template for signed JWPlayer behind akamai/cloudflare was always weak (signed direct-media -&gt; no row selectors, 1 net pattern). Recognize the signed-media + JWPlayer shape so the draft is usable.</t>
-        </is>
-      </c>
-      <c r="D10" s="13" t="inlineStr">
-        <is>
-          <t>BUILT @293; SANDBOX-VERIFIED on real WACZ @298 (corpus); live-on-stash creds pending</t>
-        </is>
-      </c>
-      <c r="E10" s="16" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="F10" s="18" t="inlineStr">
-        <is>
-          <t>Yes (recognizer unit-tested on synthetic network_log; real WACZ stash-only)</t>
+          <t>Builder enrichment slice 3 (remainder)</t>
+        </is>
+      </c>
+      <c r="D10" s="21" t="inlineStr">
+        <is>
+          <t>AWAITING OPERATOR CAPTURE DATA -- corpus-blocked remainder (build resumes after guided capture)</t>
+        </is>
+      </c>
+      <c r="E10" s="20" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F10" s="16" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
       <c r="G10" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>corpus breadth</t>
         </is>
       </c>
       <c r="H10" s="8" t="inlineStr">
         <is>
-          <t>Now verified on REAL signed-JWPlayer WACZ via the §9 corpus (reptyle/ultra/wow=wowgirls -&gt; signed_generic_token/jwplayer/pick_test_promote = R5 signing-free pattern). Remaining: live capture on stash with ultrafilms creds ('site Ultra missing password'), then flip -&gt;LIVE.</t>
+          <t>The passive dom_log trigger-derivation half shipped @258; increment-2b remains rejected. Approximately six no-rrweb-click families still need real guided picks on stash, followed by scrubbed-corpus review and builder work. The default-ON live HUD is complete and available, so HUD is no longer a dependency; only real capture breadth remains.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="11" t="inlineStr">
         <is>
-          <t>LOGIN-NSTEP</t>
+          <t>2c-DATA</t>
         </is>
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>Capture frontier</t>
+          <t>OPV / capture frontier</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>Cross-origin N-step login flow (general): plan_login_flow derivation + replay_saved_login_flow drive</t>
-        </is>
-      </c>
-      <c r="D11" s="12" t="inlineStr">
-        <is>
-          <t>BUILT @302 (code LIVE; live cross-origin DRIVE = operator-verify)</t>
-        </is>
-      </c>
-      <c r="E11" s="19" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="F11" s="17" t="inlineStr">
-        <is>
-          <t>Partial</t>
+          <t>reptyle selector re-capture -- the stored reptyle trigger matches 0 on today's live DOM; re-capture/re-review the selectors.</t>
+        </is>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>AWAITING OPERATOR (re-capture)</t>
+        </is>
+      </c>
+      <c r="E11" s="17" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="F11" s="10" t="inlineStr">
+        <is>
+          <t>No (stash/live)</t>
         </is>
       </c>
       <c r="G11" s="12" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>live reptyle DOM</t>
         </is>
       </c>
       <c r="H11" s="12" t="inlineStr">
         <is>
-          <t>login_flow_recorder.plan_login_flow derives a general N-step plan (type/click + await_url at each origin hop; single-origin = no await; credential resolves to a VAULT MARKER, never the secret, F2). replay_saved_login_flow drives it before the single-form cascade. Recorder/replay substrate (login_flow_recorder/macro_recorder/macro_replay) extended. Derivation unit-tested offline (test_v3_66_302_login_flow_nstep); live cross-origin browser drive is operator-verify on stash. FUNCTION_INDEX + DEPENDENCY_GRAPH regenerated. | Progress: 353 added staged 2-step login fill; 381 login_assist infers N-step (assist-only, cannot persist creds/enable host). Full cross-origin flow still needs operator live-verify.</t>
+          <t>Box has app.reptyle.com.candidate.json + auth.reptyle.com.template-draft.json but NOT app.reptyle.com.template-draft.json. Re-capture as part of OPV-B2.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>P3-T12-CALLSITE</t>
+          <t>CORPUS-DISPOSITION</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>Migration Phase 3-4 / capture frontier</t>
+          <t>Corpus review</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>Held-open runner call-site swap (capture_session.py) to invoke the @389 challenge seam, + on-stash live real-challenge validation before any ratchet</t>
+          <t>Manual semantic disposition of 445 draft-review-required corpus items</t>
         </is>
       </c>
       <c r="D12" s="13" t="inlineStr">
         <is>
-          <t>BUILT + DEPLOYED @458 (live real-challenge acceptance pending)</t>
-        </is>
-      </c>
-      <c r="E12" s="19" t="inlineStr">
-        <is>
-          <t>A</t>
+          <t>AWAITING OPERATOR (445 semantic reviews remain; not an OPV failure)</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="F12" s="10" t="inlineStr">
         <is>
-          <t>No (build+deploy DONE @458; live real-challenge on stash)</t>
+          <t>No (operator review)</t>
         </is>
       </c>
       <c r="G12" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Manual semantic classification of 445 review-required drafts</t>
         </is>
       </c>
       <c r="H12" s="8" t="inlineStr">
         <is>
-          <t>SHIPPED @3.66.458 (guard cut): tools/capture_session.py held-open settle call site swapped _settle_through_challenge(page) -&gt; new _settle_challenge_handoff(page), which routes through the canonical seam bulk_downloader.session_capture.handle_challenge_on_page with passive_budget_s=_challenge_wait_seconds() (budget parity) + secret-free stderr log_fn + operator_instructions() surfaced on operator_action_required. Old local poller retired; detection/passive-self-clear/manual-handoff only (no-solving static guard). GUARD SHA declared f634104a -&gt; 430f5070; other 6 byte-identical. RED-first test_p3_t12_callsite.py 5/5; build_release added=1 changed=6 removed=0 forbidden_new=0; band from extracted zip under real pytest 84 passed; verify_release --zip PASS. DEPLOYED + on-stash GREEN (10348/10289/0/59, /api/health 3.66.458). REMAINING (operator-side, not sandbox-testable): live real-challenge validation (detect-&gt;pause-&gt;handoff-&gt;detector-gated resume; solved stays False) before any ratchet.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="11" t="inlineStr">
-        <is>
-          <t>NAV</t>
-        </is>
-      </c>
-      <c r="B13" s="12" t="inlineStr">
-        <is>
-          <t>Capture frontier</t>
-        </is>
-      </c>
-      <c r="C13" s="12" t="inlineStr">
-        <is>
-          <t>Capture navigation-blocker re-test on a genuine heavy-SPA target</t>
-        </is>
-      </c>
-      <c r="D13" s="13" t="inlineStr">
-        <is>
-          <t>DIAGNOSTIC READY -- awaiting operator stash re-test</t>
-        </is>
-      </c>
-      <c r="E13" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F13" s="10" t="inlineStr">
-        <is>
-          <t>No (stash browser)</t>
-        </is>
-      </c>
-      <c r="G13" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H13" s="12" t="inlineStr">
-        <is>
-          <t>nav_probe.py 10/10 ready (built, sandbox-complete). ONLY remaining: operator runs the navigation-blocker re-test on a genuine heavy-SPA target on stash. CONDITIONAL follow-up (new item if triggered): if the probe shows N1/N3, request guard-change approval for capture_session.py and ship that fix ALONE. Nothing sandbox-buildable remains for this item itself.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t>RPTYL</t>
-        </is>
-      </c>
-      <c r="B14" s="8" t="inlineStr">
-        <is>
-          <t>Capture frontier</t>
-        </is>
-      </c>
-      <c r="C14" s="8" t="inlineStr">
-        <is>
-          <t>reptyle real-Chrome authenticated-profile capture (success = api_patterns &gt;= 1)</t>
-        </is>
-      </c>
-      <c r="D14" s="13" t="inlineStr">
-        <is>
-          <t>AWAITING OPERATOR -- real-Chrome stash capture (no sandbox build)</t>
-        </is>
-      </c>
-      <c r="E14" s="20" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="F14" s="10" t="inlineStr">
-        <is>
-          <t>No (real Chrome on stash)</t>
-        </is>
-      </c>
-      <c r="G14" s="8" t="inlineStr">
-        <is>
-          <t>HUD</t>
-        </is>
-      </c>
-      <c r="H14" s="8" t="inlineStr">
-        <is>
-          <t>First real-site capture; HUD turns it from blind to guided | No sandbox-buildable content: this is a real-site authenticated-profile capture run on stash (success = api_patterns &gt;= 1). HUD is a soft enabler (guided vs blind), not a hard prerequisite.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="11" t="inlineStr">
-        <is>
-          <t>HUD</t>
-        </is>
-      </c>
-      <c r="B15" s="12" t="inlineStr">
-        <is>
-          <t>Capture frontier</t>
-        </is>
-      </c>
-      <c r="C15" s="12" t="inlineStr">
-        <is>
-          <t>Live Capture Overlay (F2.7) live-mount half (real-time HUD during capture)</t>
-        </is>
-      </c>
-      <c r="D15" s="13" t="inlineStr">
-        <is>
-          <t>AWAITING OPERATOR -- gated on NAV re-test + guard-SHA approval before the live-mount cut</t>
-        </is>
-      </c>
-      <c r="E15" s="19" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="F15" s="10" t="inlineStr">
-        <is>
-          <t>No (stash page-wiring)</t>
-        </is>
-      </c>
-      <c r="G15" s="12" t="inlineStr">
-        <is>
-          <t>NAV re-test + guard-SHA approval</t>
-        </is>
-      </c>
-      <c r="H15" s="12" t="inlineStr">
-        <is>
-          <t>Pure half LIVE; single call site in capture_session.py (guard), default-off, fail-open. THE corpus unblocker | The live-mount guard-cut cannot honestly start in-sandbox until (a) the NAV heavy-SPA re-test determines whether a nav fix bundles in, and (b) the operator approves the capture_session.py guard-SHA change. Pure HUD half already LIVE.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="7" t="inlineStr">
-        <is>
-          <t>FR-A6.2</t>
-        </is>
-      </c>
-      <c r="B16" s="8" t="inlineStr">
-        <is>
-          <t>Capture frontier</t>
-        </is>
-      </c>
-      <c r="C16" s="8" t="inlineStr">
-        <is>
-          <t>Builder enrichment slice 2 (non-CF / non-video.js breadth)</t>
-        </is>
-      </c>
-      <c r="D16" s="21" t="inlineStr">
-        <is>
-          <t>AWAITING OPERATOR CAPTURE DATA -- corpus-blocked (build resumes after capture)</t>
-        </is>
-      </c>
-      <c r="E16" s="20" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="F16" s="18" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G16" s="8" t="inlineStr">
-        <is>
-          <t>corpus breadth</t>
-        </is>
-      </c>
-      <c r="H16" s="8" t="inlineStr">
-        <is>
-          <t>Recognition already broad; remaining breadth is guided-capture-bound | Enumerated family backlog (from the v3.66.318 KB corpus-expansion note, previously un-listed in any row): radiant_media_player, clappr, dashjs, youtube, jplayer, mux_hosted, brid_tv -- recognizer-coverage candidates for this slice / FR-A6.3 remainder. | Recognition already broad; the remaining families (radiant_media_player, clappr, dashjs, youtube, jplayer, mux_hosted, brid_tv) need operator guided captures before any recognizer breadth can be built.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="11" t="inlineStr">
-        <is>
-          <t>FR-A6.3</t>
-        </is>
-      </c>
-      <c r="B17" s="12" t="inlineStr">
-        <is>
-          <t>Capture frontier</t>
-        </is>
-      </c>
-      <c r="C17" s="12" t="inlineStr">
-        <is>
-          <t>Builder enrichment slice 3 (remainder)</t>
-        </is>
-      </c>
-      <c r="D17" s="21" t="inlineStr">
-        <is>
-          <t>AWAITING OPERATOR CAPTURE DATA -- corpus-blocked remainder (build resumes after guided capture)</t>
-        </is>
-      </c>
-      <c r="E17" s="20" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="F17" s="17" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="G17" s="12" t="inlineStr">
-        <is>
-          <t>corpus breadth</t>
-        </is>
-      </c>
-      <c r="H17" s="12" t="inlineStr">
-        <is>
-          <t>258 added dom_log passive trigger derivation. ~6 no-rrweb-click families need guided pick (HUD); increment-2b REJECTED | ~6 no-rrweb-click families need guided pick (HUD) on stash; the passive-trigger build half shipped @258.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="7" t="inlineStr">
-        <is>
-          <t>NEXT-2</t>
-        </is>
-      </c>
-      <c r="B18" s="8" t="inlineStr">
-        <is>
-          <t>Operator verify</t>
-        </is>
-      </c>
-      <c r="C18" s="8" t="inlineStr">
-        <is>
-          <t>Re-promote wowgirls cleanly via normalize_template_draft.py -&gt; promote_template.py</t>
-        </is>
-      </c>
-      <c r="D18" s="8" t="inlineStr">
-        <is>
-          <t>SANDBOX PART DONE @459 (runtime-shape gold landed; gui_parity reconciled @460) -- operator re-promote remains</t>
-        </is>
-      </c>
-      <c r="E18" s="22" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="F18" s="10" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G18" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H18" s="8" t="inlineStr">
-        <is>
-          <t>Runtime-shape GOLD shipped: tools/wow_promote_golden.py + tests/golden/wow_promote.golden.json + tests/test_wow_promote_runtime_shape.py (RED-first; the normalized candidate clears promote_gate_errors + carries the top-level resolutions ladder the raw template lacked; F2-clean). OPERATOR (on stash): re-promote wowgirls cleanly via normalize_template_draft.py -&gt; promote_template.py, then run tools/wow_promote_golden.py --check to confirm the runtime shape matches the gold. 459+460 deployed + on-stash GREEN (10355/10296/0/59).</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="11" t="inlineStr">
-        <is>
-          <t>2c-DATA</t>
-        </is>
-      </c>
-      <c r="B19" s="12" t="inlineStr">
-        <is>
-          <t>OPV / capture frontier</t>
-        </is>
-      </c>
-      <c r="C19" s="12" t="inlineStr">
-        <is>
-          <t>reptyle selector re-capture -- the stored reptyle trigger matches 0 on today's live DOM; re-capture/re-review the selectors.</t>
-        </is>
-      </c>
-      <c r="D19" s="13" t="inlineStr">
-        <is>
-          <t>AWAITING OPERATOR (re-capture)</t>
-        </is>
-      </c>
-      <c r="E19" s="16" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="F19" s="10" t="inlineStr">
-        <is>
-          <t>No (stash/live)</t>
-        </is>
-      </c>
-      <c r="G19" s="12" t="inlineStr">
-        <is>
-          <t>live reptyle DOM</t>
-        </is>
-      </c>
-      <c r="H19" s="12" t="inlineStr">
-        <is>
-          <t>Box has app.reptyle.com.candidate.json + auth.reptyle.com.template-draft.json but NOT app.reptyle.com.template-draft.json. Re-capture as part of OPV-B2.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="7" t="inlineStr">
-        <is>
-          <t>OPV-VPNKILL-LIVE</t>
-        </is>
-      </c>
-      <c r="B20" s="8" t="inlineStr">
-        <is>
-          <t>Operator verify / infrastructure</t>
-        </is>
-      </c>
-      <c r="C20" s="8" t="inlineStr">
-        <is>
-          <t>Real WireGuard tunnel fail-closed test: tunnel-down must block clear-interface egress and tunnel-up must permit expected egress.</t>
-        </is>
-      </c>
-      <c r="D20" s="13" t="inlineStr">
-        <is>
-          <t>AWAITING OPERATOR (infrastructure-bound)</t>
-        </is>
-      </c>
-      <c r="E20" s="19" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="F20" s="10" t="inlineStr">
-        <is>
-          <t>No (real tunnel on stash)</t>
-        </is>
-      </c>
-      <c r="G20" s="8" t="inlineStr">
-        <is>
-          <t>WireGuard kernel module absent on stash; real tunnel required</t>
-        </is>
-      </c>
-      <c r="H20" s="8" t="inlineStr">
-        <is>
-          <t>Keep distinct from completed OPV-VPNKILL, which proves only the sandbox/netns mechanism without a real tunnel or credentials. The July 20 OPV measurement remains BLOCKED; do not claim this live arm complete.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="11" t="inlineStr">
-        <is>
-          <t>CORPUS-DISPOSITION</t>
-        </is>
-      </c>
-      <c r="B21" s="12" t="inlineStr">
-        <is>
-          <t>Corpus review</t>
-        </is>
-      </c>
-      <c r="C21" s="12" t="inlineStr">
-        <is>
-          <t>Manual disposition of 181 review-ready drafts, 445 draft-review-required items, 3 invalid WACZ archives, and 2 JSON parse failures retained for review.</t>
-        </is>
-      </c>
-      <c r="D21" s="13" t="inlineStr">
-        <is>
-          <t>AWAITING OPERATOR (manual disposition; not an OPV failure)</t>
-        </is>
-      </c>
-      <c r="E21" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F21" s="10" t="inlineStr">
-        <is>
-          <t>No (operator review)</t>
-        </is>
-      </c>
-      <c r="G21" s="12" t="inlineStr">
-        <is>
-          <t>Manual corpus classification and archive disposition</t>
-        </is>
-      </c>
-      <c r="H21" s="12" t="inlineStr">
-        <is>
-          <t>Source: reports/OPV_VALIDATION_REPORT_2026-07-21.md. Builder and normalization processing completed 626/626; originals were not modified. These retained review populations are corpus debt, not a failed OPV acceptance lane.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="7" t="inlineStr">
-        <is>
-          <t>OPV-F2A-LIVE-CORRELATION</t>
-        </is>
-      </c>
-      <c r="B22" s="8" t="inlineStr">
-        <is>
-          <t>Operator verify / live data</t>
-        </is>
-      </c>
-      <c r="C22" s="8" t="inlineStr">
-        <is>
-          <t>F2a non-empty failure-history proof: the site-health worst-site result must correlate with the top failure cluster.</t>
-        </is>
-      </c>
-      <c r="D22" s="13" t="inlineStr">
-        <is>
-          <t>AWAITING OPERATOR (non-empty live history required)</t>
-        </is>
-      </c>
-      <c r="E22" s="15" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="F22" s="10" t="inlineStr">
-        <is>
-          <t>No (live failure history)</t>
-        </is>
-      </c>
-      <c r="G22" s="8" t="inlineStr">
-        <is>
-          <t>stash needs sanctioned, non-empty site failure history</t>
-        </is>
-      </c>
-      <c r="H22" s="8" t="inlineStr">
-        <is>
-          <t>Keep the historical OPV-F2a completed render/empty-state mechanism row intact. This distinct observation remains unexercised because the July 20 live measurement returned 0 clusters and 0 per-site rows; after sanctioned failures exist, verify the highest failure-count site appears at or near the top cluster and document any tie/recovery exception.</t>
+          <t>The technical anomaly tails are disposed safely: the three invalid WACZ entries were non-unique/sidecar cases rather than lost unique captures, and the two JSON parse anomalies were missing-tool stderr artifacts rather than corpus records. The 181 review-ready preflight rows were technically processed, but that processing is not represented as semantic approval. Operator-ready deterministic review artifacts now exist at .superpowers/sdd/corpus-disposition-review-buckets.json and .superpowers/sdd/corpus-disposition-review-buckets.md, generated by tools/corpus_disposition_buckets.py and covered by tests/test_corpus_disposition_buckets.py. They index exactly 445 unique capture-SHA rows into 8 exact gate-error buckets: 378 require selector review, 204 media/network review, and 73 resolution review (dimensions overlap). Safety posture is explicit: 0 auto-promotions, 0 artifact-secret findings, and no source paths, URLs, or queries in the artifacts. Artifact SHA-256 values: JSON 4777132e44f7466e08d803165e58d3efaf69dc2e33925eb8aaea77de62f70ed3; Markdown ff5d6730ae9b3c0d7717b00cab210b37e39ee5d2864d8e87b9340dff6afcb044. Validation passed 65 focused tests, then 103 parity/index/corpus tests after the required generated-artifact regeneration. Remaining blocker: a human must resolve each capture SHA against the private source manifest and record an explicit semantic accept/reject decision; deterministic bucketing is not semantic approval. This remains corpus debt, not a failed OPV lane.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H22"/>
+  <autoFilter ref="A1:H12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1722,7 +1294,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F273"/>
+  <dimension ref="A1:F284"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4122,7 +3694,7 @@
           <t>3.66.261 session</t>
         </is>
       </c>
-      <c r="E75" s="23" t="inlineStr">
+      <c r="E75" s="22" t="inlineStr">
         <is>
           <t>DECIDED</t>
         </is>
@@ -4218,7 +3790,7 @@
           <t>3.66.208</t>
         </is>
       </c>
-      <c r="E78" s="23" t="inlineStr">
+      <c r="E78" s="22" t="inlineStr">
         <is>
           <t>CLOSED</t>
         </is>
@@ -5434,7 +5006,7 @@
           <t>3.66.301</t>
         </is>
       </c>
-      <c r="E116" s="23" t="inlineStr">
+      <c r="E116" s="22" t="inlineStr">
         <is>
           <t>CLOSED (descoped)</t>
         </is>
@@ -8698,7 +8270,7 @@
           <t>3.66.503</t>
         </is>
       </c>
-      <c r="E218" s="23" t="inlineStr">
+      <c r="E218" s="22" t="inlineStr">
         <is>
           <t>DEPLOYED + on-stash GREEN (10693/10634/0/59)</t>
         </is>
@@ -10469,8 +10041,360 @@
         </is>
       </c>
     </row>
+    <row r="274">
+      <c r="A274" s="7" t="inlineStr">
+        <is>
+          <t>F0.4</t>
+        </is>
+      </c>
+      <c r="B274" s="8" t="inlineStr">
+        <is>
+          <t>Track-F</t>
+        </is>
+      </c>
+      <c r="C274" s="8" t="inlineStr">
+        <is>
+          <t>Production WSGI swap to waitress with SSE-compatible response headers and explicit thread sizing</t>
+        </is>
+      </c>
+      <c r="D274" s="8" t="inlineStr">
+        <is>
+          <t>v3.66.794; live-verified on v3.66.817</t>
+        </is>
+      </c>
+      <c r="E274" s="18" t="inlineStr">
+        <is>
+          <t>COMPLETED / LIVE</t>
+        </is>
+      </c>
+      <c r="F274" s="8" t="inlineStr">
+        <is>
+          <t>SHIPPED @794: downloader_ui._serve_wsgi selects waitress in production, retains werkzeug for debug/fail-open fallback, and sizes the pool with BD_WSGI_THREADS (default 30); waitress&gt;=3.0,&lt;4.0 is declared and the SSE hop-by-hop Connection header was removed. LIVE @817 on stash: installed the offline waitress 3.0.2 wheel, restarted successfully, /api/health remained ok, the response header reported Server: waitress, tests/test_v3_66_794_waitress_swap.py passed 7/7, and live L35 SSE passed 1/1 with zero warnings/failures. No systemd ExecStart rewrite was required because the production entry point invokes _serve_wsgi directly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="11" t="inlineStr">
+        <is>
+          <t>HUD</t>
+        </is>
+      </c>
+      <c r="B275" s="12" t="inlineStr">
+        <is>
+          <t>Capture frontier</t>
+        </is>
+      </c>
+      <c r="C275" s="12" t="inlineStr">
+        <is>
+          <t>Live Capture Overlay (F2.7) live mount: default-ON, persistent, CSP-immune real-time HUD during capture</t>
+        </is>
+      </c>
+      <c r="D275" s="12" t="inlineStr">
+        <is>
+          <t>v3.66.229-239; reconciled on v3.66.817</t>
+        </is>
+      </c>
+      <c r="E275" s="18" t="inlineStr">
+        <is>
+          <t>COMPLETED / LIVE</t>
+        </is>
+      </c>
+      <c r="F275" s="12" t="inlineStr">
+        <is>
+          <t>The stale NAV/guard gate was dissolved @229 and the guarded live call site shipped. @230 made the HUD default-ON, persistent across navigation, CSP-immune via page.evaluate, fail-open, and operator-toggleable; current capture_session mounts it from _pump_dom and re-mounts every tick. Actual on-stash WowGirls render confirmations are recorded @235-239, including cross-origin persistence, click/action feedback, internal scrolling, and direct-media READY parity. The measured stash service also carries BD_HUD_OVERLAY=1. No further guard approval or live-mount cut remains.</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="7" t="inlineStr">
+        <is>
+          <t>NAV</t>
+        </is>
+      </c>
+      <c r="B276" s="8" t="inlineStr">
+        <is>
+          <t>Capture frontier</t>
+        </is>
+      </c>
+      <c r="C276" s="8" t="inlineStr">
+        <is>
+          <t>Capture navigation-blocker re-test on a genuine heavy-SPA target</t>
+        </is>
+      </c>
+      <c r="D276" s="8" t="inlineStr">
+        <is>
+          <t>v3.66.817 OPV</t>
+        </is>
+      </c>
+      <c r="E276" s="18" t="inlineStr">
+        <is>
+          <t>COMPLETED (live CloakBrowser re-test)</t>
+        </is>
+      </c>
+      <c r="F276" s="8" t="inlineStr">
+        <is>
+          <t>The operator tail completed on stash against https://app.reptyle.com/ using nav_probe.probe with the configured CloakBrowser backend and the recorder attached. Result: backend=cloakbrowser, recorder_attached=true, verdict=LOAD_OK, exit 0. Per the probe contract, load reached a usable DOM, so navigation is not the blocker and no capture_session wait_until guard change is warranted. The earlier reptyle blocker was already root-caused @228-229 as stale enabled-template drift rather than page.goto behavior.</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="11" t="inlineStr">
+        <is>
+          <t>NEXT-2</t>
+        </is>
+      </c>
+      <c r="B277" s="12" t="inlineStr">
+        <is>
+          <t>Operator verify</t>
+        </is>
+      </c>
+      <c r="C277" s="12" t="inlineStr">
+        <is>
+          <t>Re-promote wowgirls cleanly through normalize_template_draft.py -&gt; promote_template.py and verify the runtime-shape golden</t>
+        </is>
+      </c>
+      <c r="D277" s="12" t="inlineStr">
+        <is>
+          <t>v3.66.817 OPV</t>
+        </is>
+      </c>
+      <c r="E277" s="18" t="inlineStr">
+        <is>
+          <t>COMPLETED (reviewed, not enabled)</t>
+        </is>
+      </c>
+      <c r="F277" s="12" t="inlineStr">
+        <is>
+          <t>Completed on stash from the preserved raw draft/review candidate with pre-change backups. The normalized candidate produced reviewed/auth.wowgirls.com.template.json with status=reviewed_not_enabled, two safe templated network patterns, and resolutions [4320, 2160, 540, 480, 360, 240]. scan_artifact_secrets returned 0 findings; tools/wow_promote_golden.py --check reported no drift; tools/validate_templates.py --root templates/reviewed returned VERDICT ok. Final template SHA-256: 3b42cca86fc993c272f3551c5a68e92626382738e2eb197cf4326641e1c53f47.</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" s="7" t="inlineStr">
+        <is>
+          <t>F2-HYG</t>
+        </is>
+      </c>
+      <c r="B278" s="8" t="inlineStr">
+        <is>
+          <t>Operator F2</t>
+        </is>
+      </c>
+      <c r="C278" s="8" t="inlineStr">
+        <is>
+          <t>Share-archive and Tiny4k WACZ hygiene: retain only canonically redacted artifacts and quarantine raw twins</t>
+        </is>
+      </c>
+      <c r="D278" s="8" t="inlineStr">
+        <is>
+          <t>v3.66.817 OPV</t>
+        </is>
+      </c>
+      <c r="E278" s="18" t="inlineStr">
+        <is>
+          <t>COMPLETED (operator-data hygiene verified)</t>
+        </is>
+      </c>
+      <c r="F278" s="8" t="inlineStr">
+        <is>
+          <t>A full Z: filename search found no redacted_captures_keep.zip, so the stale seven-raw-twins target is absent. out.zip was backed up and rebuilt through the canonical redactor with 12 redacted-only members; every member passed both artifact-secret and redaction-floor scans with 0 findings, and the rebuilt target SHA-256 is e174b2dc15da8759b569e6161ef516784035c697733098625bd39b0ab70cfa8e. Tiny4k1.redacted.wacz and Tiny4k2.redacted.wacz each passed canonical artifact/floor scans with 0 findings, and their raw twins were moved into quarantine rather than shared or deleted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" s="11" t="inlineStr">
+        <is>
+          <t>OPV-F1.4</t>
+        </is>
+      </c>
+      <c r="B279" s="12" t="inlineStr">
+        <is>
+          <t>Operator verify</t>
+        </is>
+      </c>
+      <c r="C279" s="12" t="inlineStr">
+        <is>
+          <t>F1.4 predictive_relogin on a churn-prone site -&gt; relogin at approximately 0.8 * learned median</t>
+        </is>
+      </c>
+      <c r="D279" s="12" t="inlineStr">
+        <is>
+          <t>v3.66.817 OPV</t>
+        </is>
+      </c>
+      <c r="E279" s="18" t="inlineStr">
+        <is>
+          <t>COMPLETED (live predictive relogin observed)</t>
+        </is>
+      </c>
+      <c r="F279" s="12" t="inlineStr">
+        <is>
+          <t>Live stash verification used four sanctioned churn observations with a learned median of 217.854 seconds, producing the expected 0.8 target of 174.283 seconds. One preemptive relogin occurred within the scheduler's 60-second poll cadence, reset the observed age, and did not wait for the fixed 168-hour fallback. The predictive_relogin_enabled flag was restored OFF after the measurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="7" t="inlineStr">
+        <is>
+          <t>OPV-F1.3</t>
+        </is>
+      </c>
+      <c r="B280" s="8" t="inlineStr">
+        <is>
+          <t>Operator verify</t>
+        </is>
+      </c>
+      <c r="C280" s="8" t="inlineStr">
+        <is>
+          <t>F1.3 cookie admission: an expired jar blocks worker spawn and a fresh jar self-resolves</t>
+        </is>
+      </c>
+      <c r="D280" s="8" t="inlineStr">
+        <is>
+          <t>v3.66.817 OPV</t>
+        </is>
+      </c>
+      <c r="E280" s="18" t="inlineStr">
+        <is>
+          <t>COMPLETED (live expired/fresh jar transition verified)</t>
+        </is>
+      </c>
+      <c r="F280" s="8" t="inlineStr">
+        <is>
+          <t>Live evidence is preserved at /home/mboyle/.bd21-backups/F1X-20260722T234808Z/evidence.json. With a deliberately expired dated cookie jar, admission reached cookies_expired in 1 second, retained a pending unique job, and spawned zero new browser PIDs. Restoring the original/fresh jar self-resolved the same lane to running in 2 seconds. Cleanup restored the exact pre-test config and cookie hashes and preserved queue depth 962.</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" s="11" t="inlineStr">
+        <is>
+          <t>OPV-F2A-LIVE-CORRELATION</t>
+        </is>
+      </c>
+      <c r="B281" s="12" t="inlineStr">
+        <is>
+          <t>Operator verify / live data</t>
+        </is>
+      </c>
+      <c r="C281" s="12" t="inlineStr">
+        <is>
+          <t>F2a non-empty failure-history proof: worst-site ranking correlates with the top failure cluster</t>
+        </is>
+      </c>
+      <c r="D281" s="12" t="inlineStr">
+        <is>
+          <t>v3.66.817 live hot-patch / OPV</t>
+        </is>
+      </c>
+      <c r="E281" s="18" t="inlineStr">
+        <is>
+          <t>COMPLETED (live non-empty correlation verified)</t>
+        </is>
+      </c>
+      <c r="F281" s="12" t="inlineStr">
+        <is>
+          <t>The deployed ranking fix was applied only after the remote preimage matched the local base. Focused verification passed 94 local tests and 14 dedicated on-stash tests; the service remained active under Waitress and /api/health stayed ok. The live API ranked site 48c4ddc3 first with failures=99 and score=50, while the top failure cluster named the same site with count=52; correlated=true. This closes the distinct non-empty-history observation while preserving the earlier completed empty-state/render mechanism evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="7" t="inlineStr">
+        <is>
+          <t>OPV-VPNKILL-LIVE</t>
+        </is>
+      </c>
+      <c r="B282" s="8" t="inlineStr">
+        <is>
+          <t>Operator verify / infrastructure</t>
+        </is>
+      </c>
+      <c r="C282" s="8" t="inlineStr">
+        <is>
+          <t>Real WireGuard tunnel fail-closed acceptance: tunnel-down blocks clear-interface egress and tunnel-up permits expected proxied egress</t>
+        </is>
+      </c>
+      <c r="D282" s="8" t="inlineStr">
+        <is>
+          <t>v3.66.817 OPV</t>
+        </is>
+      </c>
+      <c r="E282" s="18" t="inlineStr">
+        <is>
+          <t>COMPLETED (isolated real WireGuard acceptance)</t>
+        </is>
+      </c>
+      <c r="F282" s="8" t="inlineStr">
+        <is>
+          <t>Evidence is preserved at /home/mboyle/.bd21-backups/VPNKILL-LIVE-20260723T000017Z/evidence.json. The isolated bd-opv-local-wg tunnel completed a real WireGuard handshake and passed SOCKS/echo traffic. Killing it produced the expected killed state and exactly one callback; an idempotent repeat did not duplicate the callback. With the tunnel down, destination-scoped fail-closed nft enforcement blocked egress and its counter advanced by exactly +1. Both watchdog and manual rollback paths restored the original routes, IP state, and rules exactly. SSH and the BulkDownloader service remained available; Waitress and /api/health reported v3.66.817 healthy with queue_depth=962 and active=0. The separate API-stop link-cleanup defect was not claimed by this acceptance; it is independently closed under OPV-VPNKILL-CLEANUP.</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" s="11" t="inlineStr">
+        <is>
+          <t>OPV-VPNKILL-CLEANUP</t>
+        </is>
+      </c>
+      <c r="B283" s="12" t="inlineStr">
+        <is>
+          <t>Operator verify / infrastructure hardening</t>
+        </is>
+      </c>
+      <c r="C283" s="12" t="inlineStr">
+        <is>
+          <t>API stop teardown must remove the isolated WireGuard link after releasing runtime state and SOCKS resources</t>
+        </is>
+      </c>
+      <c r="D283" s="12" t="inlineStr">
+        <is>
+          <t>v3.66.817 live hot-patch / OPV</t>
+        </is>
+      </c>
+      <c r="E283" s="18" t="inlineStr">
+        <is>
+          <t>COMPLETED (normal API-stop ownership-scoped cleanup verified)</t>
+        </is>
+      </c>
+      <c r="F283" s="12" t="inlineStr">
+        <is>
+          <t>Evidence is preserved at /home/mboyle/.bd21-backups/VPNKILL-CLEANUP-VERIFY-20260723T001742Z/evidence.json; the deployed patch backup is /home/mboyle/.bd21-backups/VPNKILL-CLEANUP-PATCH-20260723T001550Z. Focused verification passed 113/113 tests. A normal service restart returned active/running under Waitress with /api/health ok. The isolated WireGuard start produced a nonzero handshake and successful SOCKS echo round trip. Normal API stop then removed the owned wg-bdopvlocalw link without manual deletion, closed/refused the SOCKS listener, reported state down with port 0, and removed the temporary config. Final IP addresses, routes, rules, tunnel-config SHA, and iptables/nft structure (ignoring live counters/timestamps) matched exactly; the default/LAN routes were untouched. The independent watchdog was disarmed without firing. Fresh SSH, active service, Waitress, healthy API, queue_depth=962, and active=0 confirmed the final state.</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" s="7" t="inlineStr">
+        <is>
+          <t>OPV-F3.2</t>
+        </is>
+      </c>
+      <c r="B284" s="8" t="inlineStr">
+        <is>
+          <t>Operator verify</t>
+        </is>
+      </c>
+      <c r="C284" s="8" t="inlineStr">
+        <is>
+          <t>F3.2 live drift-to-AI repair produces a disabled draft_review_required proposal and persists the run record</t>
+        </is>
+      </c>
+      <c r="D284" s="8" t="inlineStr">
+        <is>
+          <t>v3.66.817 OPV</t>
+        </is>
+      </c>
+      <c r="E284" s="18" t="inlineStr">
+        <is>
+          <t>COMPLETED (live real-Ollama repair verified)</t>
+        </is>
+      </c>
+      <c r="F284" s="8" t="inlineStr">
+        <is>
+          <t>Evidence and rollback backups are preserved at /home/mboyle/.bd21-backups/F3.2-live-20260723T000646Z. A forced API run against real Ollama qwen2.5:7b returned considered=1, repaired=1, skipped=0. The proposal had status=draft_review_required, review_required=true, enabled=false, source_capture=drift_repair:f32-opv.invalid, selector #download-video, and 0 artifact-secret findings. Draft evidence SHA-256: 9382a3030dea52d8fff56ad5655f2532c675d13dcc0a00b6e2def5ce08cb3476; persisted last-run evidence SHA-256: a22792a0fba38e97a434ccfd9d472e2e79adc0bf5c6bf5c91dba02a134603ff6. Exact rollback removed the temporary site, reset drift, removed temporary captures/draft, and restored the prior last-run record. Final state: site_count=2, temp site absent, automation disabled, drafts=8, and /api/health ok on v3.66.817 with queue_depth=962 and active=0.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F273"/>
+  <autoFilter ref="A1:F284"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -10546,7 +10470,7 @@
           <t>extraction_core Phase 1</t>
         </is>
       </c>
-      <c r="E2" s="23" t="inlineStr">
+      <c r="E2" s="22" t="inlineStr">
         <is>
           <t>REJECTED</t>
         </is>
@@ -10578,7 +10502,7 @@
           <t>247-249 era</t>
         </is>
       </c>
-      <c r="E3" s="23" t="inlineStr">
+      <c r="E3" s="22" t="inlineStr">
         <is>
           <t>REJECTED</t>
         </is>
@@ -10610,7 +10534,7 @@
           <t>3.66.247</t>
         </is>
       </c>
-      <c r="E4" s="23" t="inlineStr">
+      <c r="E4" s="22" t="inlineStr">
         <is>
           <t>DROPPED</t>
         </is>
@@ -10642,7 +10566,7 @@
           <t>3.66.318</t>
         </is>
       </c>
-      <c r="E5" s="23" t="inlineStr">
+      <c r="E5" s="22" t="inlineStr">
         <is>
           <t>DESCOPED</t>
         </is>
@@ -10674,7 +10598,7 @@
           <t>3.66.211</t>
         </is>
       </c>
-      <c r="E6" s="23" t="inlineStr">
+      <c r="E6" s="22" t="inlineStr">
         <is>
           <t>SUPERSEDED</t>
         </is>
@@ -10706,7 +10630,7 @@
           <t>permanent</t>
         </is>
       </c>
-      <c r="E7" s="23" t="inlineStr">
+      <c r="E7" s="22" t="inlineStr">
         <is>
           <t>OUT OF SCOPE</t>
         </is>
@@ -10738,7 +10662,7 @@
           <t>permanent</t>
         </is>
       </c>
-      <c r="E8" s="23" t="inlineStr">
+      <c r="E8" s="22" t="inlineStr">
         <is>
           <t>OUT OF SCOPE</t>
         </is>
@@ -10770,7 +10694,7 @@
           <t>permanent</t>
         </is>
       </c>
-      <c r="E9" s="23" t="inlineStr">
+      <c r="E9" s="22" t="inlineStr">
         <is>
           <t>OUT OF SCOPE</t>
         </is>
@@ -10802,7 +10726,7 @@
           <t>deferred-doc 2026-06-14 (v3.66.246)</t>
         </is>
       </c>
-      <c r="E10" s="23" t="inlineStr">
+      <c r="E10" s="22" t="inlineStr">
         <is>
           <t>REJECTED (do not implement)</t>
         </is>
@@ -10834,7 +10758,7 @@
           <t>v3.48+ roadmap declination</t>
         </is>
       </c>
-      <c r="E11" s="23" t="inlineStr">
+      <c r="E11" s="22" t="inlineStr">
         <is>
           <t>OUT OF SCOPE</t>
         </is>
@@ -10866,7 +10790,7 @@
           <t>3.66.502</t>
         </is>
       </c>
-      <c r="E12" s="23" t="inlineStr">
+      <c r="E12" s="22" t="inlineStr">
         <is>
           <t>PERMANENTLY DEFERRED (until necessary)</t>
         </is>

</xml_diff>

<commit_message>
chore: checkpoint code intelligence work before task 6
</commit_message>
<xml_diff>
--- a/TASK_TRACKER.xlsx
+++ b/TASK_TRACKER.xlsx
@@ -194,11 +194,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -852,12 +852,12 @@
       </c>
       <c r="G2" s="8" t="inlineStr">
         <is>
-          <t>Operator-owned MOD3 target/DSN + live shadow observability + cutover + &gt;=2-week soak</t>
+          <t>Schema/data parity + production ownership/least-privilege + durable shadow evidence + cutover + &gt;=2-week soak</t>
         </is>
       </c>
       <c r="H2" s="8" t="inlineStr">
         <is>
-          <t>The MOD3 cutover/rollback mechanism is complete @804, but it is default-OFF and tests explicitly preserve this real exit criterion. Read-only readiness audit 2026-07-22: stash has a non-empty 23-row SQLite source, psycopg, and running candidate Postgres containers, but the service has no MOD3 DSN, shadow-read, or cutover enabled; neither container is yet operator-authorized. Live shadow counters are process-local and no in-process status surface currently exposes the comparison denominator, so a separate Python preflight would not attest the running service. No clock started. Select/provision the target, add secret-free in-process stats/preflight evidence, pass rehearsal and live preflight, perform the authorized cutover, run the full on-stash suite green post-cutover, then retain &gt;=336 hours of operator-soak evidence. Exact preflight, rollback, and soak checklist: reports/OPV_EXIT3_F31_READINESS_AUDIT_2026-07-22.md.</t>
+          <t>Production target selection is complete: dedicated PostgreSQL 16 container bd-opv-postgres on loopback port 55432; the unrelated pump-tracker database was not used or changed. A rollback-safe 2026-07-23 audit preserved SQLite and target backups, proved the target dump restores, passed the isolated MOD3 suite (38 tests), and passed a bounded 23/23 history-projection rehearsal. Cutover remains correctly blocked: the source has 59 non-sqlite_% tables and 2,196 rows while the target model has six user tables and two rows; overlapping table shapes differ; live shadow recorded one divergence; preflight_cutover returned ok=false; cutover_engaged=false. No service environment, restart, production mutation, cutover, or two-week soak clock occurred. Evidence: /home/mboyle/.bd21-backups/20260723T012708Z-exit3-postgres/EXIT3_EVIDENCE_REPORT.md (SHA-256 81cb9fa1fde9a8d7b2beb7dd68ba21d15a06fb299d4e34d965418af52fa36362). Next: define the migration boundary, version the complete schema/backfill/parity gates, provision a non-superuser production-owned target, persist representative shadow evidence, then cut over only after every fail-closed gate passes and retain &gt;=336 hours of soak.</t>
         </is>
       </c>
     </row>
@@ -877,12 +877,12 @@
           <t>F3.1 enqueue lane — saved search action=enqueue -&gt; cap+gates+dedup over a week</t>
         </is>
       </c>
-      <c r="D3" s="13" t="inlineStr">
-        <is>
-          <t>AWAITING OPERATOR (week-long live verify)</t>
-        </is>
-      </c>
-      <c r="E3" s="14" t="inlineStr">
+      <c r="D3" s="12" t="inlineStr">
+        <is>
+          <t>LIVE OBSERVATION (7-day clock started 2026-07-23T01:37:15Z)</t>
+        </is>
+      </c>
+      <c r="E3" s="13" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -894,12 +894,12 @@
       </c>
       <c r="G3" s="12" t="inlineStr">
         <is>
-          <t>Operator-approved sanctioned rule + seven uninterrupted days</t>
+          <t>Seven uninterrupted days of bounded live evidence through 2026-07-30T01:37:15Z</t>
         </is>
       </c>
       <c r="H3" s="12" t="inlineStr">
         <is>
-          <t>LIVE @223; scheduler blocker cleared @461; time-warp/leak-freedom sandbox proof completed @539. Read-only readiness audit 2026-07-22 found the scheduler healthy (`saved_searches.run_due` enabled, 300-second task interval, last status ok) but zero saved-search rules, so no seven-day clock started. Operator must approve a bounded action=enqueue rule (hourly recommended), then preserve &gt;=168 hours of cap, downstream-gate, dedup, scheduler, and queue evidence. Exact rule fields and observation checklist: reports/OPV_EXIT3_F31_READINESS_AUDIT_2026-07-22.md. The deferred SPA action-picker tail remains part of this row. Consolidates former duplicate F3.1-WK.</t>
+          <t>LIVE @223; scheduler blocker cleared @461; time-warp/leak-freedom sandbox proof completed @539. The seven-day clock started at 2026-07-23T01:37:15Z using rule id 7, opv-f31-wk-fixture-20260723: fixture site only, action=enqueue, schedule=daily, daily_cap=1, notifications empty. Its first natural scheduler run at 01:39:10Z produced one new match and one enqueue from source history 26; downstream dedup finished skipped_duplicate and wrote 0 bytes. Scheduler/service/health were good, configs did not drift, and the FilthyKings queue stayed untouched at 962. Evidence: /home/mboyle/.bd21-backups/opv-f31-20260723T012540Z/RESULT.json (SHA-256 1d74f3338c78bb73754ddb3a8a4c44153b1ee4674042e60c5a86ee18d9e80d02). Keep the bounded rule unchanged and preserve daily cap, dedup, scheduler, queue, and health evidence for &gt;=168 uninterrupted hours. The deferred SPA action-picker tail remains part of this row. Consolidates former duplicate F3.1-WK.</t>
         </is>
       </c>
     </row>
@@ -919,7 +919,7 @@
           <t>Held-open capture died on anti-bot sites before the operator could act, and a login redirect dropped the deep URL onto home. A) page-death recovery; B) 'Go to my URL' re-nav; C) challenge settle.</t>
         </is>
       </c>
-      <c r="D4" s="13" t="inlineStr">
+      <c r="D4" s="14" t="inlineStr">
         <is>
           <t>LIVE A/B PASSED; challenge C pending</t>
         </is>
@@ -961,7 +961,7 @@
           <t>Auto-template for signed JWPlayer behind akamai/cloudflare was always weak (signed direct-media -&gt; no row selectors, 1 net pattern). Recognize the signed-media + JWPlayer shape so the draft is usable.</t>
         </is>
       </c>
-      <c r="D5" s="13" t="inlineStr">
+      <c r="D5" s="14" t="inlineStr">
         <is>
           <t>BUILT @293; SANDBOX-VERIFIED on real WACZ @298 (corpus); live-on-stash creds pending</t>
         </is>
@@ -1045,9 +1045,9 @@
           <t>Held-open runner call-site swap (capture_session.py) to invoke the @389 challenge seam, + on-stash live real-challenge validation before any ratchet</t>
         </is>
       </c>
-      <c r="D7" s="13" t="inlineStr">
-        <is>
-          <t>LIVE detect/pause/handoff observed; detector-gated resume pending</t>
+      <c r="D7" s="14" t="inlineStr">
+        <is>
+          <t>LIVE detect/pause/handoff + human CAPTCHA/login observed; detector-gated resume evidence pending</t>
         </is>
       </c>
       <c r="E7" s="19" t="inlineStr">
@@ -1062,12 +1062,12 @@
       </c>
       <c r="G7" s="12" t="inlineStr">
         <is>
-          <t>human clears a real challenge so detector-gated resume can be observed</t>
+          <t>an explicit detector-cleared/resume event from a real challenge run</t>
         </is>
       </c>
       <c r="H7" s="12" t="inlineStr">
         <is>
-          <t>SHIPPED @458: the held-open runner routes challenge settle through bulk_downloader.session_capture.handle_challenge_on_page with passive-budget parity, secret-free logging, operator instructions, and no solving. LIVE @817 on the real Reptyle Cloudflare login wall: the detector recognized the challenge, paused capture, routed to operator handoff, and retained solved=false. This proves the real detect-&gt;pause-&gt;handoff half. Keep the row open until a human clears a real challenge and the detector observes it gone before resume; never infer solved from the handoff itself.</t>
+          <t>SHIPPED @458: the held-open runner routes challenge settle through bulk_downloader.session_capture.handle_challenge_on_page with passive-budget parity, secret-free logging, operator instructions, and no solving. LIVE @817 on the real Reptyle Cloudflare login wall: the detector recognized the challenge, paused capture, routed to operator handoff, and retained solved=false. On 2026-07-23 the human completed the CAPTCHA and login, and the same Cloak session then captured authenticated play/download evidence. The journal preserves challenge_present and operator_action_required but no explicit detector-cleared/resume event, so this row remains open rather than inferring resume from later authenticated activity. Capture evidence: /home/mboyle/.bd21-backups/RPTYL-auth-20260723T012112Z/evidence.json.</t>
         </is>
       </c>
     </row>
@@ -1084,12 +1084,12 @@
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>reptyle real-Chrome authenticated-profile capture (success = api_patterns &gt;= 1)</t>
-        </is>
-      </c>
-      <c r="D8" s="13" t="inlineStr">
-        <is>
-          <t>AWAITING OPERATOR -- real-Chrome stash capture (no sandbox build)</t>
+          <t>Reptyle authenticated-profile runtime-browser capture (legacy success criterion = api_patterns &gt;= 1)</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>AUTHENTICATED CLOAK CAPTURE COMPLETE; legacy api_patterns&gt;=1 criterion unmet</t>
         </is>
       </c>
       <c r="E8" s="20" t="inlineStr">
@@ -1099,17 +1099,17 @@
       </c>
       <c r="F8" s="10" t="inlineStr">
         <is>
-          <t>No (real Chrome on stash)</t>
+          <t>No (persistent Cloak on stash)</t>
         </is>
       </c>
       <c r="G8" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>api_patterns=0 under the row's legacy close criterion</t>
         </is>
       </c>
       <c r="H8" s="8" t="inlineStr">
         <is>
-          <t>Run the authenticated-profile capture on stash and require api_patterns &gt;= 1. The default-ON live HUD is complete and available for guided capture, so it is no longer a blocker; this row remains open solely for the real authenticated Reptyle capture and evidence review.</t>
+          <t>Authenticated persistent-Cloak capture completed on stash: authenticated home verified, play captured, download captured, and verify tier ready. The canonical redacted WACZ is 4,191,695 bytes with two resources, zero residual secret findings, and SHA-256 c9c4a59455808798d4b7687b0c7e97f0cf66eec54d3fa1cb62a8a98fdf6be723. The high-confidence hls_manifest draft is disabled/review-only with selectors for download, login, player, quality, and settings; draft SHA-256 8d4ea97cd5e29d4fb18a28ed95750d796911ac0728f69af6d2ccd6a136360fb7. Because api_pattern_count=0, do not falsely close this legacy api_patterns&gt;=1 row. Evidence: /home/mboyle/.bd21-backups/RPTYL-auth-20260723T012112Z. Raw capture remains quarantine-only; no template was enabled or promoted.</t>
         </is>
       </c>
     </row>
@@ -1213,9 +1213,9 @@
           <t>reptyle selector re-capture -- the stored reptyle trigger matches 0 on today's live DOM; re-capture/re-review the selectors.</t>
         </is>
       </c>
-      <c r="D11" s="13" t="inlineStr">
-        <is>
-          <t>AWAITING OPERATOR (re-capture)</t>
+      <c r="D11" s="14" t="inlineStr">
+        <is>
+          <t>RE-CAPTURE COMPLETE; selector review/test pending</t>
         </is>
       </c>
       <c r="E11" s="17" t="inlineStr">
@@ -1230,12 +1230,12 @@
       </c>
       <c r="G11" s="12" t="inlineStr">
         <is>
-          <t>live reptyle DOM</t>
+          <t>review and test the five recaptured selector kinds against the live Reptyle DOM</t>
         </is>
       </c>
       <c r="H11" s="12" t="inlineStr">
         <is>
-          <t>Box has app.reptyle.com.candidate.json + auth.reptyle.com.template-draft.json but NOT app.reptyle.com.template-draft.json. Re-capture as part of OPV-B2.</t>
+          <t>The 2026-07-23 authenticated persistent-Cloak re-capture produced a high-confidence disabled/review-only draft with five selector kinds: download, login, player, quality, and settings. Play and download were captured, and the redacted WACZ has zero residual secret findings. This advances the missing/stale-selector data requirement but does not attest selector correctness: review and replay-test the five kinds before closing or promoting anything. Evidence: /home/mboyle/.bd21-backups/RPTYL-auth-20260723T012112Z; draft SHA-256 8d4ea97cd5e29d4fb18a28ed95750d796911ac0728f69af6d2ccd6a136360fb7.</t>
         </is>
       </c>
     </row>
@@ -1255,9 +1255,9 @@
           <t>Manual semantic disposition of 445 draft-review-required corpus items</t>
         </is>
       </c>
-      <c r="D12" s="13" t="inlineStr">
-        <is>
-          <t>AWAITING OPERATOR (445 semantic reviews remain; not an OPV failure)</t>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>TRIAGED 445/445; all retained review-required (not an OPV failure)</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -1272,12 +1272,12 @@
       </c>
       <c r="G12" s="8" t="inlineStr">
         <is>
-          <t>Manual semantic classification of 445 review-required drafts</t>
+          <t>Per-template review/testing before any future promotion; none are eligible for automatic enablement</t>
         </is>
       </c>
       <c r="H12" s="8" t="inlineStr">
         <is>
-          <t>The technical anomaly tails are disposed safely: the three invalid WACZ entries were non-unique/sidecar cases rather than lost unique captures, and the two JSON parse anomalies were missing-tool stderr artifacts rather than corpus records. The 181 review-ready preflight rows were technically processed, but that processing is not represented as semantic approval. Operator-ready deterministic review artifacts now exist at .superpowers/sdd/corpus-disposition-review-buckets.json and .superpowers/sdd/corpus-disposition-review-buckets.md, generated by tools/corpus_disposition_buckets.py and covered by tests/test_corpus_disposition_buckets.py. They index exactly 445 unique capture-SHA rows into 8 exact gate-error buckets: 378 require selector review, 204 media/network review, and 73 resolution review (dimensions overlap). Safety posture is explicit: 0 auto-promotions, 0 artifact-secret findings, and no source paths, URLs, or queries in the artifacts. Artifact SHA-256 values: JSON 4777132e44f7466e08d803165e58d3efaf69dc2e33925eb8aaea77de62f70ed3; Markdown ff5d6730ae9b3c0d7717b00cab210b37e39ee5d2864d8e87b9340dff6afcb044. Validation passed 65 focused tests, then 103 parity/index/corpus tests after the required generated-artifact regeneration. Remaining blocker: a human must resolve each capture SHA against the private source manifest and record an explicit semantic accept/reject decision; deterministic bucketing is not semantic approval. This remains corpus debt, not a failed OPV lane.</t>
+          <t>Safe semantic triage is complete for all 445 unique capture-SHA rows across the eight deterministic gate-error batches. Disposition for every row is retain_review_required under policy retain_review_required_non_circumvention: 445 retained, 0 rejected, 0 promoted, and 0 auto-enabled. This is an explicit safety disposition, not semantic approval of selectors, media/network patterns, resolution logic, DRM/EME handling, or site behavior. The private evidence artifact is /home/mboyle/.bd21-backups/corpus-semantic-review-445.json (424,462 bytes; SHA-256 547d5d8d281de0e995e48de436271d1df8592495a4dfae227e651e38ecee1e93). The repository's path-free eight-bucket artifacts remain .superpowers/sdd/corpus-disposition-review-buckets.json and .superpowers/sdd/corpus-disposition-review-buckets.md. Any future promotion must be based on separate review and tests; this triage made no runtime, queue, site-config, or template-enablement change.</t>
         </is>
       </c>
     </row>

</xml_diff>